<commit_message>
Import: category/subcategory column support and updated sample Excel
- ImportMapping now accepts category and subcategory column names
- enrichRows reads those columns from the uploaded file, resolves names to IDs,
  and marks rows confirmed immediately — rules/history only run as fallback
- guessMapping auto-detects Category and Subcategory columns
- Sample Excel updated with Category and Subcategory columns pre-filled

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/public/sample_statement.xlsx
+++ b/public/sample_statement.xlsx
@@ -397,13 +397,15 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E11"/>
+  <dimension ref="A1:G11"/>
   <cols>
     <col min="1" max="1" width="14.83203125" customWidth="1"/>
     <col min="2" max="2" width="42.83203125" customWidth="1"/>
     <col min="3" max="3" width="12.83203125" customWidth="1"/>
     <col min="4" max="4" width="12.83203125" customWidth="1"/>
     <col min="5" max="5" width="18.83203125" customWidth="1"/>
+    <col min="6" max="6" width="18.83203125" customWidth="1"/>
+    <col min="7" max="7" width="18.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -422,6 +424,12 @@
       <c r="E1" t="str">
         <v>Reference</v>
       </c>
+      <c r="F1" t="str">
+        <v>Category</v>
+      </c>
+      <c r="G1" t="str">
+        <v>Subcategory</v>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="str">
@@ -439,6 +447,12 @@
       <c r="E2" t="str">
         <v>SAL202407</v>
       </c>
+      <c r="F2" t="str">
+        <v>Income</v>
+      </c>
+      <c r="G2" t="str">
+        <v>Salary</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
@@ -456,6 +470,12 @@
       <c r="E3" t="str">
         <v>UPI240702001</v>
       </c>
+      <c r="F3" t="str">
+        <v>Food &amp; Dining</v>
+      </c>
+      <c r="G3" t="str">
+        <v>Food Delivery</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="str">
@@ -473,6 +493,12 @@
       <c r="E4" t="str">
         <v>AMZ240703A</v>
       </c>
+      <c r="F4" t="str">
+        <v>Shopping</v>
+      </c>
+      <c r="G4" t="str">
+        <v/>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="str">
@@ -490,6 +516,12 @@
       <c r="E5" t="str">
         <v>BESCOM07245</v>
       </c>
+      <c r="F5" t="str">
+        <v>Utilities</v>
+      </c>
+      <c r="G5" t="str">
+        <v>Electricity</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="str">
@@ -507,6 +539,12 @@
       <c r="E6" t="str">
         <v>LIC000198372</v>
       </c>
+      <c r="F6" t="str">
+        <v>Insurance</v>
+      </c>
+      <c r="G6" t="str">
+        <v>Life Insurance</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="str">
@@ -524,6 +562,12 @@
       <c r="E7" t="str">
         <v>NFLX240710</v>
       </c>
+      <c r="F7" t="str">
+        <v>Subscriptions</v>
+      </c>
+      <c r="G7" t="str">
+        <v>Streaming</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="str">
@@ -541,6 +585,12 @@
       <c r="E8" t="str">
         <v>IMPS240712001</v>
       </c>
+      <c r="F8" t="str">
+        <v/>
+      </c>
+      <c r="G8" t="str">
+        <v/>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="str">
@@ -558,6 +608,12 @@
       <c r="E9" t="str">
         <v>UPI240715009</v>
       </c>
+      <c r="F9" t="str">
+        <v>Food &amp; Dining</v>
+      </c>
+      <c r="G9" t="str">
+        <v>Food Delivery</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="str">
@@ -575,6 +631,12 @@
       <c r="E10" t="str">
         <v>NEFT240720B</v>
       </c>
+      <c r="F10" t="str">
+        <v>Income</v>
+      </c>
+      <c r="G10" t="str">
+        <v>Freelance</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="str">
@@ -592,10 +654,16 @@
       <c r="E11" t="str">
         <v>INT202407</v>
       </c>
+      <c r="F11" t="str">
+        <v>Income</v>
+      </c>
+      <c r="G11" t="str">
+        <v>Interest</v>
+      </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E11"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:G11"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>